<commit_message>
add frailty and loop diuretic use as covariates
</commit_message>
<xml_diff>
--- a/manuscript/tables/e-table-1-tte.xlsx
+++ b/manuscript/tables/e-table-1-tte.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10510"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10613"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/gwenaubrac/Desktop/newer-glp1-dementia-repkit/manuscript/tables/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9BCC957E-FC34-6B4D-BA70-8D2D24DE8B17}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3C293232-00CC-9949-9883-C3B6622177C2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="17700" xr2:uid="{609CF3B9-5A65-3C45-8EA5-C785028ABE13}"/>
   </bookViews>
@@ -59,15 +59,6 @@
     <t>Treatment strategies</t>
   </si>
   <si>
-    <t>• Diagnosis of T2D
-• No type 1 diabetes
-• No prior diagnosis for dementia
-• Diagnosis for overweight/obesity
-• BMI indicating overweight/obesity
-• No contra-indication for treatment (pancreatitis, thyroid cancer, gastroparesis)
-• No prior use of GLP-1 agonists (semaglutide, tirzepatide, liraglutide, dulaglutide, ablaglutide, exenative, or lixisenatide), SLGT2 inhibitors, DPP4 inhibitors, or sulfonylureas within 12 months</t>
-  </si>
-  <si>
     <t xml:space="preserve">For GLP-1 agonist vs SGLT2 inhibitors trial: 
 • Initiate use of semaglutide or tirzepatide
 • Initiate use of SGLT2 inhibitors
@@ -95,9 +86,6 @@
     <t>Causal contrast of interest</t>
   </si>
   <si>
-    <t>Intention-to-treat</t>
-  </si>
-  <si>
     <t>Follow-up</t>
   </si>
   <si>
@@ -133,6 +121,20 @@
   <si>
     <t>• Observational analog to intention-to-treat
 • Sensitivity analysis for observational analog to per-protocol, where individuals are censored when they discontinue or switch medications (using a 90 day grace period)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Intention-to-treat
+</t>
+  </si>
+  <si>
+    <t>• Diagnosis of T2D
+• Age ≥60 years
+• No type 1 diabetes
+• No prior diagnosis for dementia
+• Diagnosis for overweight/obesity
+• BMI indicating overweight/obesity
+• No contra-indication for treatment (pancreatitis, thyroid cancer, gastroparesis)
+• No prior use of GLP-1 agonists (semaglutide, tirzepatide, liraglutide, dulaglutide, ablaglutide, exenative, or lixisenatide), SLGT2 inhibitors, DPP4 inhibitors, or sulfonylureas within 12 months</t>
   </si>
 </sst>
 </file>
@@ -654,15 +656,15 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" ht="238" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:3" ht="255" x14ac:dyDescent="0.2">
       <c r="A2" s="3" t="s">
         <v>3</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>6</v>
+        <v>23</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
     </row>
     <row r="3" spans="1:3" ht="259" customHeight="1" x14ac:dyDescent="0.2">
@@ -670,29 +672,29 @@
         <v>5</v>
       </c>
       <c r="B3" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="C3" s="3" t="s">
         <v>7</v>
-      </c>
-      <c r="C3" s="3" t="s">
-        <v>8</v>
       </c>
     </row>
     <row r="4" spans="1:3" ht="168" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="3" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
     </row>
     <row r="5" spans="1:3" ht="17" x14ac:dyDescent="0.2">
       <c r="A5" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="B5" s="3" t="s">
         <v>10</v>
-      </c>
-      <c r="B5" s="3" t="s">
-        <v>11</v>
       </c>
       <c r="C5" s="3" t="s">
         <v>4</v>
@@ -700,35 +702,35 @@
     </row>
     <row r="6" spans="1:3" ht="244" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A6" s="3" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="C6" s="3" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
     </row>
     <row r="7" spans="1:3" ht="102" x14ac:dyDescent="0.2">
       <c r="A7" s="3" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>13</v>
+        <v>22</v>
       </c>
       <c r="C7" s="3" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
     </row>
     <row r="8" spans="1:3" ht="182" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="B8" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="B8" s="3" t="s">
+      <c r="C8" s="3" t="s">
         <v>17</v>
-      </c>
-      <c r="C8" s="3" t="s">
-        <v>19</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
update analyses to use overlap weights (rather than IPTW) as primary weighting method
</commit_message>
<xml_diff>
--- a/manuscript/tables/e-table-1-tte.xlsx
+++ b/manuscript/tables/e-table-1-tte.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/gwenaubrac/Desktop/Gwen's Documents/Work/Boston University GRA/Projects/GLP1s for AD/03_analysis/repository/newer-glp1-dementia-repkit/manuscript/tables/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3FB988AF-2C15-9F47-A06F-55B2DEBF4A78}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{01E55314-3DF0-FE40-8F8B-54451CE54B41}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="38400" windowHeight="21600" xr2:uid="{609CF3B9-5A65-3C45-8EA5-C785028ABE13}"/>
+    <workbookView xWindow="0" yWindow="600" windowWidth="38400" windowHeight="19720" xr2:uid="{609CF3B9-5A65-3C45-8EA5-C785028ABE13}"/>
   </bookViews>
   <sheets>
     <sheet name="Target Trial Emulation" sheetId="2" r:id="rId1"/>
@@ -102,15 +102,6 @@
     <t xml:space="preserve">Follow-up starts on the day of treatment assignment and ends at occurrence of the outcome, death, loss to follow-up, end of the study (December 31st, 2025) or 2 years after baseline, whichever occurs first. Time of randomization and time of treatment initiation are aligned (time 0). </t>
   </si>
   <si>
-    <t>• IPTW-weighted Kaplan-Meier estimator to obtain cumulative incidences of each streategy over 2 years of follow-up after adjusting for baseline confounders
-• IPTW-weights Cox proportional hazards models with robust variance estimators to compare the instantaneous risk of the outcome over follow-up for each strategy after adjusting for baseline confounders
-• Additional sensitivity analysis restricting to individuals with prior use of metformin</t>
-  </si>
-  <si>
-    <t>• Eligible individuals are assigned to the treatment strategy that their first medication fill is compatible with (index date). Inverse probability of treatment weights (IPTW) based on baseline covariates are used to mimic the exchangeability one would obtain from randomization.
-• Sensitivity analysis using entropy balancing weights instead of IPTW</t>
-  </si>
-  <si>
     <t>• Follow-up starts 90 days after treatment assignment to avoid reverse causality and reduce the influence of early events. Follow-is censored at occurrence of the outcome, death, loss to follow-up, end of the study (December 31st, 2025) or 2 years after baseline, whichever occurs first. Individuals who experience an event or are censored within those first 90 days are excluded from the analysis.
 • Sensitivity analyses: 1) requiring an additional 90 days of follow-up after the initial 90 days window; 2) including individuals censored within 90 days and early events.</t>
   </si>
@@ -135,6 +126,15 @@
   <si>
     <t>• Same as for the target trial. We also require at least 12 months of continuous insurance coverage prior to the index date and 90 days of continuous coverage after the index date and no prior mild cognitive impairment or neuroimaging during the 12-month baseline period. 
 • Sensitivity analysis requiring at least 6 months of continuous insurance coverage (instead of 12 months)</t>
+  </si>
+  <si>
+    <t>• Eligible individuals are assigned to the treatment strategy that their first medication fill is compatible with (index date). Overlap weighting (OW) based on baseline covariates are used to mimic the exchangeability one would obtain from randomization.
+• Sensitivity analyses using IPTW and entropy balancing weights instead of OW</t>
+  </si>
+  <si>
+    <t>• OW-weighted Kaplan-Meier estimator to obtain cumulative incidences of each streategy over 2 years of follow-up after adjusting for baseline confounders
+• OW-weights Cox proportional hazards models with robust variance estimators to compare the instantaneous risk of the outcome over follow-up for each strategy after adjusting for baseline confounders
+• Additional sensitivity analysis restricting to individuals with prior use of metformin</t>
   </si>
 </sst>
 </file>
@@ -661,10 +661,10 @@
         <v>3</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
     </row>
     <row r="3" spans="1:3" ht="259" customHeight="1" x14ac:dyDescent="0.2">
@@ -686,7 +686,7 @@
         <v>14</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>18</v>
+        <v>22</v>
       </c>
     </row>
     <row r="5" spans="1:3" ht="17" x14ac:dyDescent="0.2">
@@ -708,7 +708,7 @@
         <v>16</v>
       </c>
       <c r="C6" s="3" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
     </row>
     <row r="7" spans="1:3" ht="102" x14ac:dyDescent="0.2">
@@ -716,10 +716,10 @@
         <v>11</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="C7" s="3" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
     </row>
     <row r="8" spans="1:3" ht="182" customHeight="1" x14ac:dyDescent="0.2">
@@ -730,7 +730,7 @@
         <v>15</v>
       </c>
       <c r="C8" s="3" t="s">
-        <v>17</v>
+        <v>23</v>
       </c>
     </row>
   </sheetData>

</xml_diff>